<commit_message>
Update spreadsheet: add Tempo and apply fact-check fixes
Adds Tempo as the 11th protocol row in both Property Grid and
At a glance sheets with matching footnotes. Applies the same
fact-check updates pushed to the website: Tornado Cash OFAC
delisting, Aztec Alpha Mainnet + ~6s blocks + 4 keys, Zcash
Ledger deshielding support, and STRK20 "sub-2s" → "~2s" blocks.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/privacy_feature_grid.xlsx
+++ b/assets/privacy_feature_grid.xlsx
@@ -202,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -238,11 +238,55 @@
         <color rgb="003D3658"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="002A2640"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="002A2640"/>
+      </right>
+      <top style="thin">
+        <color rgb="002A2640"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="002A2640"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="002A2640"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="002A2640"/>
+      </right>
+      <top style="thin">
+        <color rgb="002A2640"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="002A2640"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -384,6 +428,8 @@
     <xf numFmtId="0" fontId="24" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -750,7 +796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -816,34 +862,34 @@
           <t>PRIVACY MODEL</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
+      <c r="C4" s="55" t="n"/>
+      <c r="D4" s="55" t="n"/>
+      <c r="E4" s="55" t="n"/>
+      <c r="F4" s="56" t="n"/>
       <c r="G4" s="5" t="inlineStr">
         <is>
           <t>CRYPTOGRAPHIC FOUNDATION</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="H4" s="55" t="n"/>
+      <c r="I4" s="56" t="n"/>
       <c r="J4" s="5" t="inlineStr">
         <is>
           <t>PERFORMANCE &amp; UX</t>
         </is>
       </c>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
-      <c r="M4" s="6" t="n"/>
+      <c r="K4" s="55" t="n"/>
+      <c r="L4" s="55" t="n"/>
+      <c r="M4" s="56" t="n"/>
       <c r="N4" s="5" t="inlineStr">
         <is>
           <t>ECOSYSTEM &amp; ACCESS</t>
         </is>
       </c>
-      <c r="O4" s="6" t="n"/>
-      <c r="P4" s="6" t="n"/>
-      <c r="Q4" s="6" t="n"/>
-      <c r="R4" s="6" t="n"/>
+      <c r="O4" s="55" t="n"/>
+      <c r="P4" s="55" t="n"/>
+      <c r="Q4" s="55" t="n"/>
+      <c r="R4" s="56" t="n"/>
       <c r="S4" s="4" t="n"/>
     </row>
     <row r="5" ht="40" customHeight="1">
@@ -2036,68 +2082,142 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>(✓)¹⁹</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>(✓)¹⁹</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>(✓)²⁰</t>
+        </is>
+      </c>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="O17" s="16" t="inlineStr">
+        <is>
+          <t>(✓)²²</t>
+        </is>
+      </c>
+      <c r="P17" s="17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q17" s="16" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="S17" s="19" t="inlineStr">
+        <is>
+          <t>5/17</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>✓ = full capability</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="26" t="inlineStr">
         <is>
           <t>(✓) = capability with caveats (see footnotes)</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="27" t="inlineStr">
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="27" t="inlineStr">
         <is>
           <t>– = absent or not applicable</t>
         </is>
       </c>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
-      <c r="O18" s="3" t="n"/>
-      <c r="P18" s="3" t="n"/>
-      <c r="Q18" s="3" t="n"/>
-      <c r="R18" s="3" t="n"/>
-      <c r="S18" s="3" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n"/>
+      <c r="N19" s="3" t="n"/>
+      <c r="O19" s="3" t="n"/>
+      <c r="P19" s="3" t="n"/>
+      <c r="Q19" s="3" t="n"/>
+      <c r="R19" s="3" t="n"/>
+      <c r="S19" s="3" t="n"/>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>Footnotes</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
-      <c r="O20" s="3" t="n"/>
-      <c r="P20" s="3" t="n"/>
-      <c r="Q20" s="3" t="n"/>
-      <c r="R20" s="3" t="n"/>
-      <c r="S20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="29" t="inlineStr">
-        <is>
-          <t>¹  incoming transactions only. can’t reliably view outgoing or verify balance. all-or-nothing, no per-transaction selectivity</t>
         </is>
       </c>
       <c r="B21" s="3" t="n"/>
@@ -2122,577 +2242,170 @@
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t>²  Orchard pool only (since May 2022). Sapling pool still relies on a trusted setup ceremony</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="n"/>
-      <c r="Q22" s="3" t="n"/>
-      <c r="R22" s="3" t="n"/>
-      <c r="S22" s="3" t="n"/>
+          <t>¹  incoming transactions only. can’t reliably view outgoing or verify balance. all-or-nothing, no per-transaction selectivity</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="29" t="inlineStr">
         <is>
-          <t>³  composable private/public functions exist, but within Aztec’s own nascent ecosystem. no existing DeFi protocols to compose with yet</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
-      <c r="O23" s="3" t="n"/>
-      <c r="P23" s="3" t="n"/>
-      <c r="Q23" s="3" t="n"/>
-      <c r="R23" s="3" t="n"/>
-      <c r="S23" s="3" t="n"/>
+          <t>²  Orchard pool only (since May 2022). Sapling pool still relies on a trusted setup ceremony</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>⁴  tagging mechanism requires pre-registering senders. can’t discover notes from unknown senders</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
-      <c r="O24" s="3" t="n"/>
-      <c r="P24" s="3" t="n"/>
-      <c r="Q24" s="3" t="n"/>
-      <c r="R24" s="3" t="n"/>
-      <c r="S24" s="3" t="n"/>
+          <t>³  composable private/public functions exist, but within Aztec’s own nascent ecosystem. no existing DeFi protocols to compose with yet</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t>⁵  auditor_elgamal_pubkey exists in mint config, but the entire confidential transfer feature is currently disabled on mainnet pending security audit</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="n"/>
-      <c r="O25" s="3" t="n"/>
-      <c r="P25" s="3" t="n"/>
-      <c r="Q25" s="3" t="n"/>
-      <c r="R25" s="3" t="n"/>
-      <c r="S25" s="3" t="n"/>
+          <t>⁴  tagging mechanism requires pre-registering senders. can’t discover notes from unknown senders</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
         <is>
-          <t>⁶  TFHE is lattice-based (LWE hardness assumption), considered PQ-resistant but less battle-tested than hash-based approaches</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="n"/>
-      <c r="R26" s="3" t="n"/>
-      <c r="S26" s="3" t="n"/>
+          <t>⁵  auditor_elgamal_pubkey exists in mint config, but the entire confidential transfer feature is currently disabled on mainnet pending security audit</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>⁷  confidential ERC-20s technically possible via fhEVM, but ecosystem is nascent with limited live deployments</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
-      <c r="P27" s="3" t="n"/>
-      <c r="Q27" s="3" t="n"/>
-      <c r="R27" s="3" t="n"/>
-      <c r="S27" s="3" t="n"/>
+          <t>⁶  TFHE is lattice-based (LWE hardness assumption), considered PQ-resistant but less battle-tested than hash-based approaches</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>⁸  ZK rollup architecture is inherently scalable, but currently ~1 TPS in Alpha with 36–72s block times. targeting 3–4s by end of 2026</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3" t="n"/>
-      <c r="O28" s="3" t="n"/>
-      <c r="P28" s="3" t="n"/>
-      <c r="Q28" s="3" t="n"/>
-      <c r="R28" s="3" t="n"/>
-      <c r="S28" s="3" t="n"/>
+          <t>⁷  confidential ERC-20s technically possible via fhEVM, but ecosystem is nascent with limited live deployments</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="29" t="inlineStr">
         <is>
-          <t>⁹  access-control privacy model (parties see only their part of a transaction). fundamentally different from ZK-based privacy: counterparties and validators see your data</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
-      <c r="L29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3" t="n"/>
-      <c r="O29" s="3" t="n"/>
-      <c r="P29" s="3" t="n"/>
-      <c r="Q29" s="3" t="n"/>
-      <c r="R29" s="3" t="n"/>
-      <c r="S29" s="3" t="n"/>
+          <t>⁸  ZK rollup architecture is inherently scalable, but currently ~1 TPS in Alpha Mainnet (launched March 31, 2026) with ~6s block times. targeting 3–4s by end of 2026</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
         <is>
-          <t>¹⁰  DeFi exists within Canton’s own Daml ecosystem. requires Daml, a separate smart contract language. not composable with Ethereum/Starknet DeFi</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="n"/>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3" t="n"/>
-      <c r="O30" s="3" t="n"/>
-      <c r="P30" s="3" t="n"/>
-      <c r="Q30" s="3" t="n"/>
-      <c r="R30" s="3" t="n"/>
-      <c r="S30" s="3" t="n"/>
+          <t>⁹  access-control privacy model (parties see only their part of a transaction). fundamentally different from ZK-based privacy: counterparties and validators see your data</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="29" t="inlineStr">
         <is>
-          <t>¹¹  horizontal scaling via network-of-networks. each node only processes its own transactions. claims no upper bound on TPS, but access-control privacy model</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="3" t="n"/>
-      <c r="K31" s="3" t="n"/>
-      <c r="L31" s="3" t="n"/>
-      <c r="M31" s="3" t="n"/>
-      <c r="N31" s="3" t="n"/>
-      <c r="O31" s="3" t="n"/>
-      <c r="P31" s="3" t="n"/>
-      <c r="Q31" s="3" t="n"/>
-      <c r="R31" s="3" t="n"/>
-      <c r="S31" s="3" t="n"/>
+          <t>¹⁰  DeFi exists within Canton’s own Daml ecosystem. requires Daml, a separate smart contract language. not composable with Ethereum/Starknet DeFi</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
         <is>
-          <t>¹²  mainnet since Sep 2024. USDCx with Circle launched Jan 2026. 350+ apps on testnet. but DeFi ecosystem still nascent</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="n"/>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3" t="n"/>
-      <c r="I32" s="3" t="n"/>
-      <c r="J32" s="3" t="n"/>
-      <c r="K32" s="3" t="n"/>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="n"/>
-      <c r="N32" s="3" t="n"/>
-      <c r="O32" s="3" t="n"/>
-      <c r="P32" s="3" t="n"/>
-      <c r="Q32" s="3" t="n"/>
-      <c r="R32" s="3" t="n"/>
-      <c r="S32" s="3" t="n"/>
+          <t>¹¹  horizontal scaling via network-of-networks. each node only processes its own transactions. claims no upper bound on TPS, but access-control privacy model</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="29" t="inlineStr">
         <is>
-          <t>¹³  off-chain execution model enables scalable private computation, but no composability between private applications limits real-world DeFi throughput</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="3" t="n"/>
-      <c r="K33" s="3" t="n"/>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="n"/>
-      <c r="N33" s="3" t="n"/>
-      <c r="O33" s="3" t="n"/>
-      <c r="P33" s="3" t="n"/>
-      <c r="Q33" s="3" t="n"/>
-      <c r="R33" s="3" t="n"/>
-      <c r="S33" s="3" t="n"/>
+          <t>¹²  mainnet since Sep 2024. USDCx with Circle launched Jan 2026. 350+ apps on testnet. but DeFi ecosystem still nascent</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="29" t="inlineStr">
         <is>
-          <t>¹⁴  Trezor supports Orchard shielded transactions. Ledger supports transparent Zcash only</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="n"/>
-      <c r="I34" s="3" t="n"/>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="n"/>
-      <c r="L34" s="3" t="n"/>
-      <c r="M34" s="3" t="n"/>
-      <c r="N34" s="3" t="n"/>
-      <c r="O34" s="3" t="n"/>
-      <c r="P34" s="3" t="n"/>
-      <c r="Q34" s="3" t="n"/>
-      <c r="R34" s="3" t="n"/>
-      <c r="S34" s="3" t="n"/>
+          <t>¹³  off-chain execution model enables scalable private computation, but no composability between private applications limits real-world DeFi throughput</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="29" t="inlineStr">
         <is>
-          <t>¹⁵  PXE client-side proving works but proving times still being optimized. variable depending on circuit complexity</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
-      <c r="L35" s="3" t="n"/>
-      <c r="M35" s="3" t="n"/>
-      <c r="N35" s="3" t="n"/>
-      <c r="O35" s="3" t="n"/>
-      <c r="P35" s="3" t="n"/>
-      <c r="Q35" s="3" t="n"/>
-      <c r="R35" s="3" t="n"/>
-      <c r="S35" s="3" t="n"/>
+          <t>¹⁴  Trezor supports Orchard shielded transactions. Ledger now supports deshielding from the Orchard pool (shielded-to-transparent spends); shielding and shielded-to-shielded sends are still Trezor-only</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="29" t="inlineStr">
         <is>
-          <t>¹⁶  can outsource to Prover Market (Proof-as-a-Service). client-side proving possible but resource-intensive</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
-      <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="3" t="n"/>
-      <c r="K36" s="3" t="n"/>
-      <c r="L36" s="3" t="n"/>
-      <c r="M36" s="3" t="n"/>
-      <c r="N36" s="3" t="n"/>
-      <c r="O36" s="3" t="n"/>
-      <c r="P36" s="3" t="n"/>
-      <c r="Q36" s="3" t="n"/>
-      <c r="R36" s="3" t="n"/>
-      <c r="S36" s="3" t="n"/>
+          <t>¹⁵  PXE client-side proving works but proving times still being optimized. variable depending on circuit complexity</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="29" t="inlineStr">
         <is>
-          <t>¹⁷  Ledger supports Solana but confidential transfer feature is currently disabled on mainnet</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
-      <c r="J37" s="3" t="n"/>
-      <c r="K37" s="3" t="n"/>
-      <c r="L37" s="3" t="n"/>
-      <c r="M37" s="3" t="n"/>
-      <c r="N37" s="3" t="n"/>
-      <c r="O37" s="3" t="n"/>
-      <c r="P37" s="3" t="n"/>
-      <c r="Q37" s="3" t="n"/>
-      <c r="R37" s="3" t="n"/>
-      <c r="S37" s="3" t="n"/>
+          <t>¹⁶  can outsource to Prover Market (Proof-as-a-Service). client-side proving possible but resource-intensive</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="29" t="inlineStr">
         <is>
-          <t>¹⁸  Orchard proofs ~2–5s on modern hardware, but limited to simple shielded transfer logic</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3" t="n"/>
-      <c r="I38" s="3" t="n"/>
-      <c r="J38" s="3" t="n"/>
-      <c r="K38" s="3" t="n"/>
-      <c r="L38" s="3" t="n"/>
-      <c r="M38" s="3" t="n"/>
-      <c r="N38" s="3" t="n"/>
-      <c r="O38" s="3" t="n"/>
-      <c r="P38" s="3" t="n"/>
-      <c r="Q38" s="3" t="n"/>
-      <c r="R38" s="3" t="n"/>
-      <c r="S38" s="3" t="n"/>
+          <t>¹⁷  Ledger supports Solana but confidential transfer feature is currently disabled on mainnet</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="29" t="inlineStr">
         <is>
-          <t>¹⁹  Bulletproofs+ for amount hiding are formally ZK, but core sender privacy relies on ring signatures which are a different cryptographic mechanism</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="n"/>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="N39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n"/>
-      <c r="Q39" s="3" t="n"/>
-      <c r="R39" s="3" t="n"/>
-      <c r="S39" s="3" t="n"/>
+          <t>¹⁸  Orchard proofs ~2–5s on modern hardware, but limited to simple shielded transfer logic</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="29" t="inlineStr">
         <is>
-          <t>²⁰  Bulletproofs for range proofs are formally ZK, but scope is limited to amount hiding only</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="n"/>
-      <c r="L40" s="3" t="n"/>
-      <c r="M40" s="3" t="n"/>
-      <c r="N40" s="3" t="n"/>
-      <c r="O40" s="3" t="n"/>
-      <c r="P40" s="3" t="n"/>
-      <c r="Q40" s="3" t="n"/>
-      <c r="R40" s="3" t="n"/>
-      <c r="S40" s="3" t="n"/>
+          <t>¹⁹  Tempo: sub-second finality on the base layer (Simplex BFT), but private transaction speed not separately benchmarked. mainnet launched March 18, 2026</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="29" t="inlineStr">
         <is>
-          <t>²¹  always private by default. no shielding needed (instant opt-in), but no way to opt-out to a transparent state</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
-      <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
-      <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="n"/>
-      <c r="L41" s="3" t="n"/>
-      <c r="M41" s="3" t="n"/>
-      <c r="N41" s="3" t="n"/>
-      <c r="O41" s="3" t="n"/>
-      <c r="P41" s="3" t="n"/>
-      <c r="Q41" s="3" t="n"/>
-      <c r="R41" s="3" t="n"/>
-      <c r="S41" s="3" t="n"/>
+          <t>²⁰  Tempo: base layer targets 100K+ TPS on Reth execution, but private transaction throughput not separately disclosed</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="29" t="inlineStr">
         <is>
-          <t>²²  1-hour mandatory standby period after shielding before funds can be used privately (Private Proof of Innocence requirement)</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
-      <c r="H42" s="3" t="n"/>
-      <c r="I42" s="3" t="n"/>
-      <c r="J42" s="3" t="n"/>
-      <c r="K42" s="3" t="n"/>
-      <c r="L42" s="3" t="n"/>
-      <c r="M42" s="3" t="n"/>
-      <c r="N42" s="3" t="n"/>
-      <c r="O42" s="3" t="n"/>
-      <c r="P42" s="3" t="n"/>
-      <c r="Q42" s="3" t="n"/>
-      <c r="R42" s="3" t="n"/>
-      <c r="S42" s="3" t="n"/>
+          <t>²¹  always private by default. no shielding needed (instant opt-in), but no way to opt-out to a transparent state</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="29" t="inlineStr">
         <is>
-          <t>²³  36–72s block times in Alpha. shielding speed will improve as block times target 3–4s by late 2026</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="3" t="n"/>
-      <c r="L43" s="3" t="n"/>
-      <c r="M43" s="3" t="n"/>
-      <c r="N43" s="3" t="n"/>
-      <c r="O43" s="3" t="n"/>
-      <c r="P43" s="3" t="n"/>
-      <c r="Q43" s="3" t="n"/>
-      <c r="R43" s="3" t="n"/>
-      <c r="S43" s="3" t="n"/>
+          <t>²²  Tempo: major design partners (Stripe, Visa, Mastercard, Deutsche Bank, Anthropic, OpenAI) but mainnet just launched March 18, 2026 — live ecosystem still nascent</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="29" t="inlineStr">
         <is>
+          <t>²³  ~6s block times in Alpha Mainnet since March 31, 2026. shielding speed will improve as block times target 3–4s by late 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="29" t="inlineStr">
+        <is>
           <t>²⁴  ~5s end-to-end from user perspective, but proof runs on wallet operator backend (48-core machine). Zcash Zashi generates proofs directly on mobile in ~5s. for an apples-to-apples comparison, proof generation is not yet on consumer hardware. mobile proving on the roadmap</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n"/>
-      <c r="C44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n"/>
-      <c r="I44" s="3" t="n"/>
-      <c r="J44" s="3" t="n"/>
-      <c r="K44" s="3" t="n"/>
-      <c r="L44" s="3" t="n"/>
-      <c r="M44" s="3" t="n"/>
-      <c r="N44" s="3" t="n"/>
-      <c r="O44" s="3" t="n"/>
-      <c r="P44" s="3" t="n"/>
-      <c r="Q44" s="3" t="n"/>
-      <c r="R44" s="3" t="n"/>
-      <c r="S44" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="30">
@@ -2763,7 +2476,6 @@
           <t>PRIVACY MODEL</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="31" t="inlineStr">
@@ -2797,7 +2509,7 @@
       </c>
       <c r="B5" s="32" t="inlineStr">
         <is>
-          <t>users handle a single signing key (or none, via AA). no per-note secrets to manage or lose. STRK20s derives all keys from the Starknet account key via account abstraction. Aztec requires 3 separate key pairs. Aleo requires private key + view key. Railgun requires spending + viewing keys. Monero requires spend + view keys. Canton uses party keys managed via validator nodes. Others also require dedicated privacy key management.</t>
+          <t>users handle a single signing key (or none, via AA). no per-note secrets to manage or lose. STRK20s derives all keys from the Starknet account key via account abstraction. Aztec requires 4 separate key pairs. Aleo requires private key + view key. Railgun requires spending + viewing keys. Monero requires spend + view keys. Canton uses party keys managed via validator nodes. Others also require dedicated privacy key management.</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2543,6 @@
           <t>CRYPTOGRAPHIC FOUNDATION</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="31" t="inlineStr">
@@ -2875,7 +2586,6 @@
           <t>PERFORMANCE &amp; UX</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
@@ -2885,7 +2595,7 @@
       </c>
       <c r="B13" s="32" t="inlineStr">
         <is>
-          <t>how quickly a user can move between public and private states. measures the end-to-end time from initiating a shield (opt-in to privacy) or unshield (opt-out) to having usable funds. STRK20s: sub-2s block confirmation + sub-5s proof generation = seconds to shield or unshield. fastest of any protocol. Zcash: ~75s block time is the bottleneck. proof generation 2–5s but must wait for block confirmation. Monero: always private by default (instant opt-in), but no way to opt-out to a transparent state. Aztec: 36–72s block times in Alpha (targeting 3–4s by late 2026). Railgun: Ethereum block time (~12s) for the on-chain tx, but a mandatory 1-hour standby period after shielding before funds can be used (Private Proof of Innocence requirement). Tornado Cash: deposit was one Ethereum block, but real privacy required waiting hours for anonymity set to build. Aleo: off-chain proving but no concrete shielding speed benchmarks available. Solana: feature disabled on mainnet. Canton: access control model, no shielding concept. Zama: FHE operations are orders of magnitude slower than ZK.</t>
+          <t>how quickly a user can move between public and private states. measures the end-to-end time from initiating a shield (opt-in to privacy) or unshield (opt-out) to having usable funds. STRK20s: ~2s block confirmation + sub-5s proof generation = seconds to shield or unshield. fastest of any protocol. Zcash: ~75s block time is the bottleneck. proof generation 2–5s but must wait for block confirmation. Monero: always private by default (instant opt-in), but no way to opt-out to a transparent state. Aztec: ~6s block times in Alpha Mainnet since March 31, 2026 (targeting 3–4s by late 2026). Railgun: Ethereum block time (~12s) for the on-chain tx, but a mandatory 1-hour standby period after shielding before funds can be used (Private Proof of Innocence requirement). Tornado Cash: deposit was one Ethereum block, but real privacy required waiting hours for anonymity set to build. Aleo: off-chain proving but no concrete shielding speed benchmarks available. Solana: feature disabled on mainnet. Canton: access control model, no shielding concept. Zama: FHE operations are orders of magnitude slower than ZK.</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2619,7 @@
       </c>
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>high throughput and low cost for private operations specifically. Starknet: ~1,000 TPS today, targeting 10k+. sub-2s confirmation, $0.002 avg fee. Canton: claims no upper bound on TPS via horizontal scaling but access-control privacy model. Aleo: off-chain execution model is architecturally scalable but no composability between private apps limits real-world DeFi throughput. Zcash: PoW L1, ~75s blocks. Monero: PoW L1, 2-min blocks. Aztec: ~1 TPS in Alpha, 36–72s blocks. Railgun: inherits L1 gas costs. Solana: fast but privacy feature disabled. Zama: FHE is orders of magnitude slower. Tornado Cash: L1 gas costs.</t>
+          <t>high throughput and low cost for private operations specifically. Starknet: ~1,000 TPS today, targeting 10k+. ~2s confirmation, $0.002 avg fee. Canton: claims no upper bound on TPS via horizontal scaling but access-control privacy model. Aleo: off-chain execution model is architecturally scalable but no composability between private apps limits real-world DeFi throughput. Zcash: PoW L1, ~75s blocks. Monero: PoW L1, 2-min blocks. Aztec: ~1 TPS in Alpha Mainnet since March 31, 2026, ~6s blocks. Railgun: inherits L1 gas costs. Solana: fast but privacy feature disabled. Zama: FHE is orders of magnitude slower. Tornado Cash: L1 gas costs.</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2641,6 @@
           <t>ECOSYSTEM &amp; ACCESS</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="31" t="inlineStr">
@@ -3011,7 +2720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3528,57 +3237,81 @@
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>(✓)¹⁸</t>
+        </is>
+      </c>
+      <c r="C16" s="42" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>(✓)¹⁹</t>
+        </is>
+      </c>
+      <c r="E16" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F16" s="41" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G16" s="42" t="inlineStr">
+        <is>
+          <t>(✓)²⁰</t>
+        </is>
+      </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>✓ = yes</t>
-        </is>
-      </c>
+      <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n"/>
-      <c r="C17" s="26" t="inlineStr">
-        <is>
-          <t>(✓) = partially (see footnotes)</t>
-        </is>
-      </c>
+      <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
-      <c r="F17" s="27" t="inlineStr">
-        <is>
-          <t>– = no</t>
-        </is>
-      </c>
+      <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>✓ = yes</t>
+        </is>
+      </c>
       <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>(✓) = partially (see footnotes)</t>
+        </is>
+      </c>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>– = no</t>
+        </is>
+      </c>
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
-        <is>
-          <t>Footnotes</t>
-        </is>
-      </c>
+      <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
@@ -3589,18 +3322,24 @@
       <c r="I19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
-        <is>
-          <t>¹  Starknet has full AA and wallet integration (Braavos, Argent), but STRK20s privacy transactions are not yet available on hardware wallets</t>
-        </is>
-      </c>
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Footnotes</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="29" t="inlineStr">
         <is>
-          <t>²  formally ZK proofs, but single-asset only (ZEC), no multi-asset pool, poor note discovery UX</t>
+          <t>¹  Starknet has full AA and wallet integration (Braavos, Argent), but STRK20s privacy transactions are not yet available on hardware wallets</t>
         </is>
       </c>
       <c r="H21" s="3" t="n"/>
@@ -3609,7 +3348,7 @@
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t>³  Trezor supports Orchard shielded transactions. Ledger only transparent</t>
+          <t>²  formally ZK proofs, but single-asset only (ZEC), no multi-asset pool, poor note discovery UX</t>
         </is>
       </c>
       <c r="H22" s="3" t="n"/>
@@ -3618,7 +3357,7 @@
     <row r="23">
       <c r="A23" s="29" t="inlineStr">
         <is>
-          <t>⁴  always-on privacy with strongest anonymity set, but no multi-asset pool, no formal ZK proofs, no secretless design</t>
+          <t>³  Trezor supports Orchard shielded transactions. Ledger now supports deshielding from the Orchard pool but not shielding or shielded-to-shielded sends</t>
         </is>
       </c>
       <c r="H23" s="3" t="n"/>
@@ -3627,7 +3366,7 @@
     <row r="24">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>⁵  incoming viewing keys only. can’t reliably verify outgoing or balance</t>
+          <t>⁴  always-on privacy with strongest anonymity set, but no multi-asset pool, no formal ZK proofs, no secretless design</t>
         </is>
       </c>
       <c r="H24" s="3" t="n"/>
@@ -3636,7 +3375,7 @@
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t>⁶  Ledger supports full shielded transactions, but no account abstraction</t>
+          <t>⁵  incoming viewing keys only. can’t reliably verify outgoing or balance</t>
         </is>
       </c>
       <c r="H25" s="3" t="n"/>
@@ -3645,7 +3384,7 @@
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
         <is>
-          <t>⁷  smart contracts exist but zero existing DeFi or liquidity. cold start problem</t>
+          <t>⁶  Ledger supports full shielded transactions, but no account abstraction</t>
         </is>
       </c>
       <c r="H26" s="3" t="n"/>
@@ -3654,7 +3393,7 @@
     <row r="27">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>⁸  PLONK uses universal SRS (still a setup). no post-quantum. but has succinct verifiability</t>
+          <t>⁷  Alpha Mainnet since March 31, 2026 — smart contracts live but DeFi ecosystem still bootstrapping. cold start problem</t>
         </is>
       </c>
       <c r="H27" s="3" t="n"/>
@@ -3663,7 +3402,7 @@
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>⁹  native AA, but no hardware wallet support for privacy transactions</t>
+          <t>⁸  PLONK uses universal SRS (still a setup). no post-quantum. but has succinct verifiability</t>
         </is>
       </c>
       <c r="H28" s="3" t="n"/>
@@ -3672,7 +3411,7 @@
     <row r="29">
       <c r="A29" s="29" t="inlineStr">
         <is>
-          <t>¹⁰  formally ZK but no multi-asset pool, no composability between private apps, no note discovery</t>
+          <t>⁹  native AA, but no hardware wallet support for privacy transactions</t>
         </is>
       </c>
       <c r="H29" s="3" t="n"/>
@@ -3681,7 +3420,7 @@
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
         <is>
-          <t>¹¹  formally ZK and multi-asset, but privacy limited by pool size per token. no client-side proving of complex logic</t>
+          <t>¹⁰  formally ZK but no multi-asset pool, no composability between private apps, no note discovery</t>
         </is>
       </c>
       <c r="H30" s="3" t="n"/>
@@ -3690,7 +3429,7 @@
     <row r="31">
       <c r="A31" s="29" t="inlineStr">
         <is>
-          <t>¹²  auditor key exists in config but entire feature is disabled on mainnet</t>
+          <t>¹¹  formally ZK and multi-asset, but privacy limited by pool size per token. no client-side proving of complex logic</t>
         </is>
       </c>
       <c r="H31" s="3" t="n"/>
@@ -3699,7 +3438,7 @@
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
         <is>
-          <t>¹³  DeFi within own Daml ecosystem only. requires separate smart contract language</t>
+          <t>¹²  auditor key exists in config but entire feature is disabled on mainnet</t>
         </is>
       </c>
       <c r="H32" s="3" t="n"/>
@@ -3708,7 +3447,7 @@
     <row r="33">
       <c r="A33" s="29" t="inlineStr">
         <is>
-          <t>¹⁴  TFHE is lattice-based (PQ-resistant) and no trusted setup, but no succinct verifiability</t>
+          <t>¹³  DeFi within own Daml ecosystem only. requires separate smart contract language</t>
         </is>
       </c>
       <c r="H33" s="3" t="n"/>
@@ -3717,7 +3456,7 @@
     <row r="34">
       <c r="A34" s="29" t="inlineStr">
         <is>
-          <t>¹⁵  formally ZK (Groth16), but fragmented pools (fixed denominations), timing analysis could de-anonymize users, and protocol is OFAC-sanctioned/defunct</t>
+          <t>¹⁴  TFHE is lattice-based (PQ-resistant) and no trusted setup, but no succinct verifiability</t>
         </is>
       </c>
       <c r="H34" s="3" t="n"/>
@@ -3726,7 +3465,7 @@
     <row r="35">
       <c r="A35" s="29" t="inlineStr">
         <is>
-          <t>¹⁶  FHE genuinely encrypts data during computation, but server-side model (not client-side ZK proofs). different trust model. ecosystem nascent</t>
+          <t>¹⁵  formally ZK (Groth16), but fragmented pools (fixed denominations) and timing analysis could de-anonymize users. protocol is defunct; OFAC sanctions were lifted in March 2025</t>
         </is>
       </c>
       <c r="H35" s="3" t="n"/>
@@ -3735,53 +3474,45 @@
     <row r="36">
       <c r="A36" s="29" t="inlineStr">
         <is>
-          <t>¹⁷  privacy is always on so there’s no shielding step (zero friction to opt in). ~2 min block time for confirmations. seamless UX but slower than Starknet</t>
+          <t>¹⁶  FHE genuinely encrypts data during computation, but server-side model (not client-side ZK proofs). different trust model. ecosystem nascent</t>
         </is>
       </c>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n"/>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>¹⁷  privacy is always on so there’s no shielding step (zero friction to opt in). ~2 min block time for confirmations. seamless UX but slower than Starknet</t>
+        </is>
+      </c>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n"/>
-      <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="n"/>
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>¹⁸  Tempo: opt-in privacy, not private by default. privacy cryptography not publicly documented. uses TIP-403 Policy Registry for issuer compliance and auditability</t>
+        </is>
+      </c>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n"/>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>¹⁹  Tempo: sub-second finality on base layer via Simplex BFT consensus, but private transaction speed not separately benchmarked</t>
+        </is>
+      </c>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n"/>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>²⁰  Tempo: native account abstraction with passkeys (P256) and MetaMask at launch, but no hardware wallet path published for confidential transfers</t>
+        </is>
+      </c>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
     </row>
@@ -4016,15 +3747,29 @@
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="n"/>
     </row>
+    <row r="62">
+      <c r="A62" s="3" t="n"/>
+      <c r="B62" s="3" t="n"/>
+      <c r="C62" s="3" t="n"/>
+      <c r="D62" s="3" t="n"/>
+      <c r="E62" s="3" t="n"/>
+      <c r="F62" s="3" t="n"/>
+      <c r="G62" s="3" t="n"/>
+      <c r="H62" s="3" t="n"/>
+      <c r="I62" s="3" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="22">
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A30:G30"/>

</xml_diff>